<commit_message>
v114: Professional Excel template with data validation dropdowns - dropdowns now prevent invalid input for Resultado and Score fields
</commit_message>
<xml_diff>
--- a/Calendario_Resultados_IMPORT.xlsx
+++ b/Calendario_Resultados_IMPORT.xlsx
@@ -1,46 +1,72 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\VSCode-Teste\taca-manuel-andre-2026\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9F06EF1-FEE7-496D-B918-A497AD68C407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{10675F78-CB6A-440C-B28A-69CCAE6A1B3B}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="InstruÃ§Ãµes" sheetId="2" r:id="rId1"/>
-    <sheet name="Resultados" sheetId="1" r:id="rId2"/>
-  </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>Calendario</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="114">
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Orlando Manuel Leite</dc:creator>
+  <cp:lastModifiedBy>Orlando Manuel Leite</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T16:46:22Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T16:46:30Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Enabled">
+    <vt:lpwstr>true</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_SetDate">
+    <vt:lpwstr>2026-07-23T16:46:30Z</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Method">
+    <vt:lpwstr>Standard</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="5" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Name">
+    <vt:lpwstr>1680d606-3385-4829-a27a-d391e7785643</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="6" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_SiteId">
+    <vt:lpwstr>b6f420c1-da14-4124-b666-fadafb6ebc04</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="7" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ActionId">
+    <vt:lpwstr>9664c3d8-75e0-42dd-ab50-8f06d1f87d2d</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="8" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ContentBits">
+    <vt:lpwstr>0</vt:lpwstr>
+  </property>
+  <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="9" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Tag">
+    <vt:lpwstr>10, 3, 0, 1</vt:lpwstr>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="98">
   <si>
     <t>matchId</t>
   </si>
@@ -334,72 +360,19 @@
   </si>
   <si>
     <t>R5-2-71</t>
-  </si>
-  <si>
-    <t>TACA MANUEL ANDRE 2026 - IMPORTACAO DE RESULTADOS</t>
-  </si>
-  <si>
-    <t>[INFO] Preenchimento:</t>
-  </si>
-  <si>
-    <t>1. Preencha APENAS as colunas 'Resultado' e 'Score (X&amp;Y)'</t>
-  </si>
-  <si>
-    <t>2. As outras colunas sao de REFERENCIA (nao edite)</t>
-  </si>
-  <si>
-    <t>[INFO] Valores validos para Resultado:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Vence A (Equipa de casa vence)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Vence B (Equipa visitante vence)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - A/S (Empate - All Square)</t>
-  </si>
-  <si>
-    <t>[INFO] Formato para Score:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - X&amp;Y onde X=pontos casa, Y=pontos fora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Exemplos: 2&amp;1, 1&amp;0, 3&amp;2</t>
-  </si>
-  <si>
-    <t>[INFO] Como exportar para CSV:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   1. Preencha os resultados e scores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   2. Guarde o ficheiro Excel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   3. Execute: Export-CSVDoExcel.ps1 (script incluido)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   4. Importe na app (Admin - Configuracoes)</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Montserrat"/>
     </font>
     <font>
       <b/>
@@ -415,12 +388,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF595959"/>
-      <name val="Montserrat"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF784E1F"/>
       <name val="Montserrat"/>
     </font>
   </fonts>
@@ -450,7 +417,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -458,29 +425,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,7 +478,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -813,113 +793,47 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{283F98B7-FE36-4253-B8AF-09D78FACC392}">
-  <dimension ref="A1:A20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="80.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="7"/>
-    </row>
-    <row r="3" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A3" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A6" s="7"/>
-    </row>
-    <row r="7" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A9" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A10" s="7" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A11" s="7"/>
-    </row>
-    <row r="12" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A12" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A13" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A14" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A15" s="7"/>
-    </row>
-    <row r="16" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A17" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A18" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A19" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A20" s="6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\VSCode-Teste\taca-manuel-andre-2026\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{943AA208-AE70-4A2A-846A-28BECCFDC578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80E0EF84-E237-4809-8F69-B51CD88F08B9}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Calendario" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
+  </extLst>
+</workbook>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6AD429C-EBDD-4F11-B068-094AD877860D}">
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{663DEC49-E9EB-4C94-869A-64DB926460F0}">
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -929,6 +843,14 @@
     <col min="4" max="5" width="22.6328125" customWidth="1"/>
     <col min="6" max="7" width="15.6328125" customWidth="1"/>
   </cols>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="F2:F9">
+      <formula1>"Vence A,Vence B,A/S"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="G2:G9">
+      <formula1>"1&amp;0,1&amp;1,1&amp;2,1&amp;3,2&amp;0,2&amp;1,2&amp;2,2&amp;3,3&amp;0,3&amp;1,3&amp;2,3&amp;3"</formula1>
+    </dataValidation>
+  </dataValidations>
   <sheetData>
     <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Fix: regenerate Excel with correct data validation ranges (F2:F73, G2:G73)
</commit_message>
<xml_diff>
--- a/Calendario_Resultados_IMPORT.xlsx
+++ b/Calendario_Resultados_IMPORT.xlsx
@@ -31,8 +31,8 @@
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <dc:creator>Orlando Manuel Leite</dc:creator>
   <cp:lastModifiedBy>Orlando Manuel Leite</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T16:46:22Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T16:46:30Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T16:59:24Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T16:59:30Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -42,7 +42,7 @@
     <vt:lpwstr>true</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_SetDate">
-    <vt:lpwstr>2026-07-23T16:46:30Z</vt:lpwstr>
+    <vt:lpwstr>2026-07-23T16:59:30Z</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Method">
     <vt:lpwstr>Standard</vt:lpwstr>
@@ -54,7 +54,7 @@
     <vt:lpwstr>b6f420c1-da14-4124-b666-fadafb6ebc04</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="7" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ActionId">
-    <vt:lpwstr>9664c3d8-75e0-42dd-ab50-8f06d1f87d2d</vt:lpwstr>
+    <vt:lpwstr>aa69f119-49db-4e8a-b7ff-6aed28656c4c</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="8" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ContentBits">
     <vt:lpwstr>0</vt:lpwstr>
@@ -366,7 +366,7 @@
 
 <file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,14 +381,11 @@
       <name val="Montserrat"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Montserrat"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FF595959"/>
-      <name val="Montserrat"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -449,16 +446,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -802,9 +797,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\VSCode-Teste\taca-manuel-andre-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{943AA208-AE70-4A2A-846A-28BECCFDC578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E5B1AB1-1F04-4503-9909-0AF94E584A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80E0EF84-E237-4809-8F69-B51CD88F08B9}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{106E3C1E-A7EA-472F-A205-BDE58A3A355A}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
@@ -833,7 +828,7 @@
 </file>
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{663DEC49-E9EB-4C94-869A-64DB926460F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F9B273-8DE2-43D3-9074-D6E2621C2D61}">
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -844,10 +839,10 @@
     <col min="6" max="7" width="15.6328125" customWidth="1"/>
   </cols>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="F2:F9">
+    <dataValidation xmlns="" type="list" allowBlank="1" showDropDown="1" sqref="F2:F73">
       <formula1>"Vence A,Vence B,A/S"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="G2:G9">
+    <dataValidation xmlns="" type="list" allowBlank="1" showDropDown="1" sqref="G2:G73">
       <formula1>"1&amp;0,1&amp;1,1&amp;2,1&amp;3,2&amp;0,2&amp;1,2&amp;2,2&amp;3,3&amp;0,3&amp;1,3&amp;2,3&amp;3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -875,7 +870,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -894,7 +889,7 @@
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -913,7 +908,7 @@
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -932,7 +927,7 @@
       <c r="F4" s="5"/>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
@@ -951,7 +946,7 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -970,7 +965,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="7" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -989,7 +984,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -1008,7 +1003,7 @@
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -1027,7 +1022,7 @@
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
     </row>
-    <row r="10" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1046,7 +1041,7 @@
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
     </row>
-    <row r="11" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -1065,7 +1060,7 @@
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -1084,7 +1079,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
     </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -1103,7 +1098,7 @@
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1122,7 +1117,7 @@
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
@@ -1141,7 +1136,7 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -1160,7 +1155,7 @@
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>
-    <row r="17" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
@@ -1179,7 +1174,7 @@
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
     </row>
-    <row r="18" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
@@ -1198,7 +1193,7 @@
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
     </row>
-    <row r="19" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
@@ -1217,7 +1212,7 @@
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
@@ -1236,7 +1231,7 @@
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
     </row>
-    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
@@ -1255,7 +1250,7 @@
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
     </row>
-    <row r="22" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
@@ -1274,7 +1269,7 @@
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
     </row>
-    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
@@ -1293,7 +1288,7 @@
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
     </row>
-    <row r="24" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
@@ -1312,7 +1307,7 @@
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
     </row>
-    <row r="25" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>45</v>
       </c>
@@ -1331,7 +1326,7 @@
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
     </row>
-    <row r="26" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>46</v>
       </c>
@@ -1350,7 +1345,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
     </row>
-    <row r="27" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>48</v>
       </c>
@@ -1369,7 +1364,7 @@
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
     </row>
-    <row r="28" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>49</v>
       </c>
@@ -1388,7 +1383,7 @@
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
     </row>
-    <row r="29" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>50</v>
       </c>
@@ -1407,7 +1402,7 @@
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
     </row>
-    <row r="30" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>51</v>
       </c>
@@ -1426,7 +1421,7 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
     </row>
-    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>53</v>
       </c>
@@ -1445,7 +1440,7 @@
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
     </row>
-    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>54</v>
       </c>
@@ -1464,7 +1459,7 @@
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
     </row>
-    <row r="33" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>55</v>
       </c>
@@ -1483,7 +1478,7 @@
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
     </row>
-    <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>56</v>
       </c>
@@ -1502,7 +1497,7 @@
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
     </row>
-    <row r="35" spans="1:7" ht="30" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>57</v>
       </c>
@@ -1521,7 +1516,7 @@
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
     </row>
-    <row r="36" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>58</v>
       </c>
@@ -1540,7 +1535,7 @@
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
     </row>
-    <row r="37" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>59</v>
       </c>
@@ -1559,7 +1554,7 @@
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
     </row>
-    <row r="38" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>60</v>
       </c>
@@ -1578,7 +1573,7 @@
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
     </row>
-    <row r="39" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>61</v>
       </c>
@@ -1597,7 +1592,7 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
     </row>
-    <row r="40" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>62</v>
       </c>
@@ -1616,7 +1611,7 @@
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
     </row>
-    <row r="41" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>63</v>
       </c>
@@ -1635,7 +1630,7 @@
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
     </row>
-    <row r="42" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>64</v>
       </c>
@@ -1654,7 +1649,7 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
     </row>
-    <row r="43" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>65</v>
       </c>
@@ -1673,7 +1668,7 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
     </row>
-    <row r="44" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>66</v>
       </c>
@@ -1692,7 +1687,7 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
     </row>
-    <row r="45" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>67</v>
       </c>
@@ -1711,7 +1706,7 @@
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
     </row>
-    <row r="46" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>68</v>
       </c>
@@ -1730,7 +1725,7 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
     </row>
-    <row r="47" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>69</v>
       </c>
@@ -1749,7 +1744,7 @@
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
     </row>
-    <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>70</v>
       </c>
@@ -1768,7 +1763,7 @@
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
     </row>
-    <row r="49" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>71</v>
       </c>
@@ -1787,7 +1782,7 @@
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
     </row>
-    <row r="50" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>72</v>
       </c>
@@ -1806,7 +1801,7 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
     </row>
-    <row r="51" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>74</v>
       </c>
@@ -1825,7 +1820,7 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
     </row>
-    <row r="52" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>75</v>
       </c>
@@ -1844,7 +1839,7 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
     </row>
-    <row r="53" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>76</v>
       </c>
@@ -1863,7 +1858,7 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
     </row>
-    <row r="54" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>77</v>
       </c>
@@ -1882,7 +1877,7 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
     </row>
-    <row r="55" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>78</v>
       </c>
@@ -1901,7 +1896,7 @@
       <c r="F55" s="5"/>
       <c r="G55" s="5"/>
     </row>
-    <row r="56" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>79</v>
       </c>
@@ -1920,7 +1915,7 @@
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
     </row>
-    <row r="57" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>80</v>
       </c>
@@ -1939,7 +1934,7 @@
       <c r="F57" s="5"/>
       <c r="G57" s="5"/>
     </row>
-    <row r="58" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>81</v>
       </c>
@@ -1958,7 +1953,7 @@
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
     </row>
-    <row r="59" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>83</v>
       </c>
@@ -1977,7 +1972,7 @@
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
     </row>
-    <row r="60" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>84</v>
       </c>
@@ -1996,7 +1991,7 @@
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
     </row>
-    <row r="61" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>85</v>
       </c>
@@ -2015,7 +2010,7 @@
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
     </row>
-    <row r="62" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>86</v>
       </c>
@@ -2034,7 +2029,7 @@
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
     </row>
-    <row r="63" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>87</v>
       </c>
@@ -2053,7 +2048,7 @@
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
     </row>
-    <row r="64" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>88</v>
       </c>
@@ -2072,7 +2067,7 @@
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
     </row>
-    <row r="65" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>89</v>
       </c>
@@ -2091,7 +2086,7 @@
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
     </row>
-    <row r="66" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>90</v>
       </c>
@@ -2110,7 +2105,7 @@
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
     </row>
-    <row r="67" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>91</v>
       </c>
@@ -2129,7 +2124,7 @@
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
     </row>
-    <row r="68" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>92</v>
       </c>
@@ -2148,7 +2143,7 @@
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
     </row>
-    <row r="69" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>93</v>
       </c>
@@ -2167,7 +2162,7 @@
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
     </row>
-    <row r="70" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>94</v>
       </c>
@@ -2186,7 +2181,7 @@
       <c r="F70" s="5"/>
       <c r="G70" s="5"/>
     </row>
-    <row r="71" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>95</v>
       </c>
@@ -2205,7 +2200,7 @@
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
     </row>
-    <row r="72" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>96</v>
       </c>
@@ -2224,7 +2219,7 @@
       <c r="F72" s="5"/>
       <c r="G72" s="5"/>
     </row>
-    <row r="73" spans="1:7" ht="15" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>97</v>
       </c>

</xml_diff>

<commit_message>
Fix: completely rebuild Excel template - clean structure with proper validation dropdowns (F2:F73, G2:G73)
</commit_message>
<xml_diff>
--- a/Calendario_Resultados_IMPORT.xlsx
+++ b/Calendario_Resultados_IMPORT.xlsx
@@ -31,8 +31,8 @@
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <dc:creator>Orlando Manuel Leite</dc:creator>
   <cp:lastModifiedBy>Orlando Manuel Leite</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T16:59:24Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T16:59:30Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T17:02:42Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T17:02:54Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -42,7 +42,7 @@
     <vt:lpwstr>true</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_SetDate">
-    <vt:lpwstr>2026-07-23T16:59:30Z</vt:lpwstr>
+    <vt:lpwstr>2026-07-23T17:02:52Z</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Method">
     <vt:lpwstr>Standard</vt:lpwstr>
@@ -54,7 +54,7 @@
     <vt:lpwstr>b6f420c1-da14-4124-b666-fadafb6ebc04</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="7" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ActionId">
-    <vt:lpwstr>aa69f119-49db-4e8a-b7ff-6aed28656c4c</vt:lpwstr>
+    <vt:lpwstr>b964c6bb-ad95-43e0-a288-b1c43aa34406</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="8" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ContentBits">
     <vt:lpwstr>0</vt:lpwstr>
@@ -378,7 +378,9 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Montserrat"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -441,18 +443,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -797,9 +795,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\VSCode-Teste\taca-manuel-andre-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E5B1AB1-1F04-4503-9909-0AF94E584A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D14ECCD0-7DD8-42E2-AB37-740DE7F6BBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{106E3C1E-A7EA-472F-A205-BDE58A3A355A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D97B40D8-DC5A-4FBC-84D8-783F8C863EDA}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
@@ -828,7 +826,7 @@
 </file>
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F9B273-8DE2-43D3-9074-D6E2621C2D61}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12104361-F1BC-4324-9B22-5DFD2A81E5D5}">
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -839,15 +837,15 @@
     <col min="6" max="7" width="15.6328125" customWidth="1"/>
   </cols>
   <dataValidations>
-    <dataValidation xmlns="" type="list" allowBlank="1" showDropDown="1" sqref="F2:F73">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="F2:F73">
       <formula1>"Vence A,Vence B,A/S"</formula1>
     </dataValidation>
-    <dataValidation xmlns="" type="list" allowBlank="1" showDropDown="1" sqref="G2:G73">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" sqref="G2:G73">
       <formula1>"1&amp;0,1&amp;1,1&amp;2,1&amp;3,2&amp;0,2&amp;1,2&amp;2,2&amp;3,3&amp;0,3&amp;1,3&amp;2,3&amp;3"</formula1>
     </dataValidation>
   </dataValidations>
   <sheetData>
-    <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -874,1369 +872,1369 @@
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3">
-        <v>2</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3">
-        <v>1</v>
-      </c>
-      <c r="C6" s="3">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3">
-        <v>1</v>
-      </c>
-      <c r="C7" s="3">
-        <v>2</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="3">
-        <v>1</v>
-      </c>
-      <c r="C8" s="3">
-        <v>1</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="3">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3">
-        <v>2</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="3">
-        <v>1</v>
-      </c>
-      <c r="C10" s="3">
-        <v>1</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="B10" s="2">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="3">
-        <v>1</v>
-      </c>
-      <c r="C11" s="3">
-        <v>2</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="3">
-        <v>1</v>
-      </c>
-      <c r="C12" s="3">
-        <v>1</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="B12" s="2">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="3">
-        <v>1</v>
-      </c>
-      <c r="C13" s="3">
-        <v>2</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="2">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="3">
-        <v>2</v>
-      </c>
-      <c r="C14" s="3">
-        <v>1</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="B14" s="2">
+        <v>2</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="3">
-        <v>2</v>
-      </c>
-      <c r="C15" s="3">
-        <v>2</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="2">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="3">
-        <v>2</v>
-      </c>
-      <c r="C16" s="3">
-        <v>1</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="B16" s="2">
+        <v>2</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="3">
-        <v>2</v>
-      </c>
-      <c r="C17" s="3">
-        <v>2</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="B17" s="2">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2">
+        <v>2</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="3">
-        <v>2</v>
-      </c>
-      <c r="C18" s="3">
-        <v>1</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="B18" s="2">
+        <v>2</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="3">
-        <v>2</v>
-      </c>
-      <c r="C19" s="3">
-        <v>2</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="B19" s="2">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2">
+        <v>2</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="3">
-        <v>2</v>
-      </c>
-      <c r="C20" s="3">
-        <v>1</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="B20" s="2">
+        <v>2</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="3">
-        <v>2</v>
-      </c>
-      <c r="C21" s="3">
-        <v>2</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="B21" s="2">
+        <v>2</v>
+      </c>
+      <c r="C21" s="2">
+        <v>2</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="3">
-        <v>2</v>
-      </c>
-      <c r="C22" s="3">
-        <v>1</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="B22" s="2">
+        <v>2</v>
+      </c>
+      <c r="C22" s="2">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="3">
-        <v>2</v>
-      </c>
-      <c r="C23" s="3">
-        <v>2</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="B23" s="2">
+        <v>2</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="2">
         <v>3</v>
       </c>
-      <c r="C24" s="3">
-        <v>1</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25" s="2">
         <v>3</v>
       </c>
-      <c r="C25" s="3">
-        <v>2</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="2">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26" s="2">
         <v>3</v>
       </c>
-      <c r="C26" s="3">
-        <v>1</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="2">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B27" s="2">
         <v>3</v>
       </c>
-      <c r="C27" s="3">
-        <v>2</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="2">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28" s="2">
         <v>3</v>
       </c>
-      <c r="C28" s="3">
-        <v>1</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="2">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29" s="2">
         <v>3</v>
       </c>
-      <c r="C29" s="3">
-        <v>2</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="2">
+        <v>2</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30" s="2">
         <v>3</v>
       </c>
-      <c r="C30" s="3">
-        <v>1</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="2">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B31" s="2">
         <v>3</v>
       </c>
-      <c r="C31" s="3">
-        <v>2</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="2">
+        <v>2</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="3">
+      <c r="B32" s="2">
         <v>3</v>
       </c>
-      <c r="C32" s="3">
-        <v>1</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="C32" s="2">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="2">
         <v>3</v>
       </c>
-      <c r="C33" s="3">
-        <v>2</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="C33" s="2">
+        <v>2</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="3">
+      <c r="B34" s="2">
         <v>3</v>
       </c>
-      <c r="C34" s="3">
-        <v>1</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="C34" s="2">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B35" s="2">
         <v>3</v>
       </c>
-      <c r="C35" s="3">
-        <v>2</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="C35" s="2">
+        <v>2</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B36" s="3">
+      <c r="B36" s="2">
         <v>4</v>
       </c>
-      <c r="C36" s="3">
-        <v>1</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="C36" s="2">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="3">
+      <c r="B37" s="2">
         <v>4</v>
       </c>
-      <c r="C37" s="3">
-        <v>2</v>
-      </c>
-      <c r="D37" s="4" t="s">
+      <c r="C37" s="2">
+        <v>2</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B38" s="3">
+      <c r="B38" s="2">
         <v>4</v>
       </c>
-      <c r="C38" s="3">
-        <v>1</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B39" s="2">
         <v>4</v>
       </c>
-      <c r="C39" s="3">
-        <v>2</v>
-      </c>
-      <c r="D39" s="4" t="s">
+      <c r="C39" s="2">
+        <v>2</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="3">
+      <c r="B40" s="2">
         <v>4</v>
       </c>
-      <c r="C40" s="3">
-        <v>1</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="C40" s="2">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B41" s="3">
+      <c r="B41" s="2">
         <v>4</v>
       </c>
-      <c r="C41" s="3">
-        <v>2</v>
-      </c>
-      <c r="D41" s="4" t="s">
+      <c r="C41" s="2">
+        <v>2</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="E41" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B42" s="3">
+      <c r="B42" s="2">
         <v>4</v>
       </c>
-      <c r="C42" s="3">
-        <v>1</v>
-      </c>
-      <c r="D42" s="4" t="s">
+      <c r="C42" s="2">
+        <v>1</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B43" s="2">
         <v>4</v>
       </c>
-      <c r="C43" s="3">
-        <v>2</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="C43" s="2">
+        <v>2</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B44" s="2">
         <v>5</v>
       </c>
-      <c r="C44" s="3">
-        <v>1</v>
-      </c>
-      <c r="D44" s="4" t="s">
+      <c r="C44" s="2">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B45" s="2">
         <v>5</v>
       </c>
-      <c r="C45" s="3">
-        <v>2</v>
-      </c>
-      <c r="D45" s="4" t="s">
+      <c r="C45" s="2">
+        <v>2</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E45" s="4" t="s">
+      <c r="E45" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B46" s="2">
         <v>5</v>
       </c>
-      <c r="C46" s="3">
-        <v>1</v>
-      </c>
-      <c r="D46" s="4" t="s">
+      <c r="C46" s="2">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E46" s="4" t="s">
+      <c r="E46" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B47" s="3">
+      <c r="B47" s="2">
         <v>5</v>
       </c>
-      <c r="C47" s="3">
-        <v>2</v>
-      </c>
-      <c r="D47" s="4" t="s">
+      <c r="C47" s="2">
+        <v>2</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B48" s="2">
         <v>5</v>
       </c>
-      <c r="C48" s="3">
-        <v>1</v>
-      </c>
-      <c r="D48" s="4" t="s">
+      <c r="C48" s="2">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="E48" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B49" s="2">
         <v>5</v>
       </c>
-      <c r="C49" s="3">
-        <v>2</v>
-      </c>
-      <c r="D49" s="4" t="s">
+      <c r="C49" s="2">
+        <v>2</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="E49" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B50" s="3">
-        <v>1</v>
-      </c>
-      <c r="C50" s="3">
-        <v>1</v>
-      </c>
-      <c r="D50" s="4" t="s">
+      <c r="B50" s="2">
+        <v>1</v>
+      </c>
+      <c r="C50" s="2">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E50" s="4" t="s">
+      <c r="E50" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B51" s="3">
-        <v>1</v>
-      </c>
-      <c r="C51" s="3">
-        <v>2</v>
-      </c>
-      <c r="D51" s="4" t="s">
+      <c r="B51" s="2">
+        <v>1</v>
+      </c>
+      <c r="C51" s="2">
+        <v>2</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E51" s="4" t="s">
+      <c r="E51" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B52" s="3">
-        <v>2</v>
-      </c>
-      <c r="C52" s="3">
-        <v>1</v>
-      </c>
-      <c r="D52" s="4" t="s">
+      <c r="B52" s="2">
+        <v>2</v>
+      </c>
+      <c r="C52" s="2">
+        <v>1</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E52" s="4" t="s">
+      <c r="E52" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B53" s="3">
-        <v>2</v>
-      </c>
-      <c r="C53" s="3">
-        <v>2</v>
-      </c>
-      <c r="D53" s="4" t="s">
+      <c r="B53" s="2">
+        <v>2</v>
+      </c>
+      <c r="C53" s="2">
+        <v>2</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E53" s="4" t="s">
+      <c r="E53" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B54" s="2">
         <v>4</v>
       </c>
-      <c r="C54" s="3">
-        <v>1</v>
-      </c>
-      <c r="D54" s="4" t="s">
+      <c r="C54" s="2">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E54" s="4" t="s">
+      <c r="E54" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B55" s="2">
         <v>4</v>
       </c>
-      <c r="C55" s="3">
-        <v>2</v>
-      </c>
-      <c r="D55" s="4" t="s">
+      <c r="C55" s="2">
+        <v>2</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E55" s="4" t="s">
+      <c r="E55" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B56" s="3">
+      <c r="B56" s="2">
         <v>5</v>
       </c>
-      <c r="C56" s="3">
-        <v>1</v>
-      </c>
-      <c r="D56" s="4" t="s">
+      <c r="C56" s="2">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E56" s="4" t="s">
+      <c r="E56" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B57" s="3">
+      <c r="B57" s="2">
         <v>5</v>
       </c>
-      <c r="C57" s="3">
-        <v>2</v>
-      </c>
-      <c r="D57" s="4" t="s">
+      <c r="C57" s="2">
+        <v>2</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E57" s="4" t="s">
+      <c r="E57" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F57" s="5"/>
-      <c r="G57" s="5"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B58" s="3">
-        <v>1</v>
-      </c>
-      <c r="C58" s="3">
-        <v>1</v>
-      </c>
-      <c r="D58" s="4" t="s">
+      <c r="B58" s="2">
+        <v>1</v>
+      </c>
+      <c r="C58" s="2">
+        <v>1</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E58" s="4" t="s">
+      <c r="E58" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F58" s="5"/>
-      <c r="G58" s="5"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B59" s="3">
-        <v>1</v>
-      </c>
-      <c r="C59" s="3">
-        <v>2</v>
-      </c>
-      <c r="D59" s="4" t="s">
+      <c r="B59" s="2">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2">
+        <v>2</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E59" s="4" t="s">
+      <c r="E59" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B60" s="3">
-        <v>2</v>
-      </c>
-      <c r="C60" s="3">
-        <v>1</v>
-      </c>
-      <c r="D60" s="4" t="s">
+      <c r="B60" s="2">
+        <v>2</v>
+      </c>
+      <c r="C60" s="2">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E60" s="4" t="s">
+      <c r="E60" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B61" s="3">
-        <v>2</v>
-      </c>
-      <c r="C61" s="3">
-        <v>2</v>
-      </c>
-      <c r="D61" s="4" t="s">
+      <c r="B61" s="2">
+        <v>2</v>
+      </c>
+      <c r="C61" s="2">
+        <v>2</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E61" s="4" t="s">
+      <c r="E61" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F61" s="5"/>
-      <c r="G61" s="5"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B62" s="2">
         <v>3</v>
       </c>
-      <c r="C62" s="3">
-        <v>1</v>
-      </c>
-      <c r="D62" s="4" t="s">
+      <c r="C62" s="2">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E62" s="4" t="s">
+      <c r="E62" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B63" s="3">
+      <c r="B63" s="2">
         <v>3</v>
       </c>
-      <c r="C63" s="3">
-        <v>2</v>
-      </c>
-      <c r="D63" s="4" t="s">
+      <c r="C63" s="2">
+        <v>2</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E63" s="4" t="s">
+      <c r="E63" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B64" s="3">
+      <c r="B64" s="2">
         <v>4</v>
       </c>
-      <c r="C64" s="3">
-        <v>1</v>
-      </c>
-      <c r="D64" s="4" t="s">
+      <c r="C64" s="2">
+        <v>1</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E64" s="4" t="s">
+      <c r="E64" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F64" s="5"/>
-      <c r="G64" s="5"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B65" s="3">
+      <c r="B65" s="2">
         <v>4</v>
       </c>
-      <c r="C65" s="3">
-        <v>2</v>
-      </c>
-      <c r="D65" s="4" t="s">
+      <c r="C65" s="2">
+        <v>2</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E65" s="4" t="s">
+      <c r="E65" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B66" s="3">
-        <v>2</v>
-      </c>
-      <c r="C66" s="3">
-        <v>1</v>
-      </c>
-      <c r="D66" s="4" t="s">
+      <c r="B66" s="2">
+        <v>2</v>
+      </c>
+      <c r="C66" s="2">
+        <v>1</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E66" s="4" t="s">
+      <c r="E66" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B67" s="3">
-        <v>2</v>
-      </c>
-      <c r="C67" s="3">
-        <v>2</v>
-      </c>
-      <c r="D67" s="4" t="s">
+      <c r="B67" s="2">
+        <v>2</v>
+      </c>
+      <c r="C67" s="2">
+        <v>2</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E67" s="4" t="s">
+      <c r="E67" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B68" s="3">
+      <c r="B68" s="2">
         <v>5</v>
       </c>
-      <c r="C68" s="3">
-        <v>1</v>
-      </c>
-      <c r="D68" s="4" t="s">
+      <c r="C68" s="2">
+        <v>1</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E68" s="4" t="s">
+      <c r="E68" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B69" s="3">
+      <c r="B69" s="2">
         <v>5</v>
       </c>
-      <c r="C69" s="3">
-        <v>2</v>
-      </c>
-      <c r="D69" s="4" t="s">
+      <c r="C69" s="2">
+        <v>2</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E69" s="4" t="s">
+      <c r="E69" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B70" s="3">
+      <c r="B70" s="2">
         <v>3</v>
       </c>
-      <c r="C70" s="3">
-        <v>1</v>
-      </c>
-      <c r="D70" s="4" t="s">
+      <c r="C70" s="2">
+        <v>1</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E70" s="4" t="s">
+      <c r="E70" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B71" s="3">
+      <c r="B71" s="2">
         <v>3</v>
       </c>
-      <c r="C71" s="3">
-        <v>2</v>
-      </c>
-      <c r="D71" s="4" t="s">
+      <c r="C71" s="2">
+        <v>2</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E71" s="4" t="s">
+      <c r="E71" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B72" s="3">
+      <c r="B72" s="2">
         <v>5</v>
       </c>
-      <c r="C72" s="3">
-        <v>1</v>
-      </c>
-      <c r="D72" s="4" t="s">
+      <c r="C72" s="2">
+        <v>1</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E72" s="4" t="s">
+      <c r="E72" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B73" s="2">
         <v>5</v>
       </c>
-      <c r="C73" s="3">
-        <v>2</v>
-      </c>
-      <c r="D73" s="4" t="s">
+      <c r="C73" s="2">
+        <v>2</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E73" s="4" t="s">
+      <c r="E73" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F73" s="5"/>
-      <c r="G73" s="5"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: regenerate clean Excel template with working validation (v115 final)
</commit_message>
<xml_diff>
--- a/Calendario_Resultados_IMPORT.xlsx
+++ b/Calendario_Resultados_IMPORT.xlsx
@@ -31,8 +31,8 @@
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <dc:creator>Orlando Manuel Leite</dc:creator>
   <cp:lastModifiedBy>Orlando Manuel Leite</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T17:02:42Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T17:02:54Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-07-23T21:25:59Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T21:26:13Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -42,7 +42,7 @@
     <vt:lpwstr>true</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="3" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_SetDate">
-    <vt:lpwstr>2026-07-23T17:02:52Z</vt:lpwstr>
+    <vt:lpwstr>2026-07-23T21:26:13Z</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="4" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_Method">
     <vt:lpwstr>Standard</vt:lpwstr>
@@ -54,7 +54,7 @@
     <vt:lpwstr>b6f420c1-da14-4124-b666-fadafb6ebc04</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="7" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ActionId">
-    <vt:lpwstr>b964c6bb-ad95-43e0-a288-b1c43aa34406</vt:lpwstr>
+    <vt:lpwstr>08d0222f-158f-4b07-a68d-6843fe825f24</vt:lpwstr>
   </property>
   <property fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="8" name="MSIP_Label_1680d606-3385-4829-a27a-d391e7785643_ContentBits">
     <vt:lpwstr>0</vt:lpwstr>
@@ -795,9 +795,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\VSCode-Teste\taca-manuel-andre-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D14ECCD0-7DD8-42E2-AB37-740DE7F6BBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A7F13F5-F1D3-41F4-A4CB-E582ADCC258E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D97B40D8-DC5A-4FBC-84D8-783F8C863EDA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{213A8B01-9E02-48E8-B671-B9B173F93BCB}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
@@ -826,7 +826,7 @@
 </file>
 
 <file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12104361-F1BC-4324-9B22-5DFD2A81E5D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B381C6-AE4A-4D9C-881F-3DCA8999C4A5}">
   <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
fix: sort calendar by ronda/grupo/home/par - Excel now ordered correctly
</commit_message>
<xml_diff>
--- a/Calendario_Resultados_IMPORT.xlsx
+++ b/Calendario_Resultados_IMPORT.xlsx
@@ -44,16 +44,40 @@
     <t xml:space="preserve">R1-1-2</t>
   </si>
   <si>
+    <t xml:space="preserve">Os Craques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os Últimos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-2-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Equipa Eleven</t>
   </si>
   <si>
     <t xml:space="preserve">EMJC</t>
   </si>
   <si>
-    <t xml:space="preserve">R1-2-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-4</t>
+    <t xml:space="preserve">R1-2-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green Legends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V.T.F.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-2-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-8</t>
   </si>
   <si>
     <t xml:space="preserve">Birdies e Boggies</t>
@@ -62,10 +86,10 @@
     <t xml:space="preserve">Jacaré</t>
   </si>
   <si>
-    <t xml:space="preserve">R1-2-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-6</t>
+    <t xml:space="preserve">R1-2-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-10</t>
   </si>
   <si>
     <t xml:space="preserve">Os Golfinhos</t>
@@ -74,10 +98,22 @@
     <t xml:space="preserve">Piratas</t>
   </si>
   <si>
-    <t xml:space="preserve">R1-2-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-8</t>
+    <t xml:space="preserve">R1-2-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golfistas da Madrugada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old Fashion Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-2-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1-1-14</t>
   </si>
   <si>
     <t xml:space="preserve">MMLH</t>
@@ -86,211 +122,175 @@
     <t xml:space="preserve">School</t>
   </si>
   <si>
-    <t xml:space="preserve">R1-2-9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Golfistas da Madrugada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Old Fashion Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-2-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Os Craques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V.T.F.</t>
+    <t xml:space="preserve">R1-2-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CGGG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-22</t>
   </si>
   <si>
     <t xml:space="preserve">Red Hot Chilli Putters</t>
   </si>
   <si>
-    <t xml:space="preserve">R2-2-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-22</t>
+    <t xml:space="preserve">R2-2-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-1-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R2-2-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-32</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">R3-2-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CGGG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-32</t>
-  </si>
-  <si>
     <t xml:space="preserve">R3-2-33</t>
   </si>
   <si>
-    <t xml:space="preserve">R4-1-34</t>
+    <t xml:space="preserve">R3-1-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-1-46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3-2-47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-48</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>
   </si>
   <si>
-    <t xml:space="preserve">R4-2-35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-1-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-2-37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-1-38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-2-39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-1-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-2-41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-1-42</t>
+    <t xml:space="preserve">R4-2-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-2-51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-2-53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-2-55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-2-57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-1-58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4-2-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-1-60</t>
   </si>
   <si>
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">R5-2-43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-1-44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-2-45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-1-46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-2-47</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Os Últimos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-2-49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-1-52</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-2-53</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-1-54</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R5-2-55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-1-56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green Legends</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1-2-57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-58</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-59</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-1-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-61</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-1-62</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R4-2-63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-1-64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R2-2-65</t>
+    <t xml:space="preserve">R5-2-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-1-62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-2-63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-1-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-2-65</t>
   </si>
   <si>
     <t xml:space="preserve">R5-1-66</t>
@@ -299,10 +299,10 @@
     <t xml:space="preserve">R5-2-67</t>
   </si>
   <si>
-    <t xml:space="preserve">R3-1-68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R3-2-69</t>
+    <t xml:space="preserve">R5-1-68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5-2-69</t>
   </si>
   <si>
     <t xml:space="preserve">R5-1-70</t>
@@ -670,7 +670,7 @@
         <v>33</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s" s="2">
         <v>8</v>
@@ -679,17 +679,17 @@
         <v>34</v>
       </c>
       <c r="E14" t="s" s="2">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C15" t="s" s="2">
         <v>12</v>
@@ -698,52 +698,52 @@
         <v>34</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C16" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E16" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s" s="2">
         <v>39</v>
-      </c>
-      <c r="B17" t="s" s="2">
-        <v>12</v>
-      </c>
-      <c r="C17" t="s" s="2">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="E17" t="s" s="2">
-        <v>38</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B18" t="s" s="2">
         <v>12</v>
@@ -752,17 +752,17 @@
         <v>8</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s" s="2">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B19" t="s" s="2">
         <v>12</v>
@@ -771,17 +771,17 @@
         <v>12</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>12</v>
@@ -790,17 +790,17 @@
         <v>8</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s" s="2">
         <v>12</v>
@@ -809,17 +809,17 @@
         <v>12</v>
       </c>
       <c r="D21" t="s" s="2">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E21" t="s" s="2">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s" s="2">
         <v>12</v>
@@ -828,17 +828,17 @@
         <v>8</v>
       </c>
       <c r="D22" t="s" s="2">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E22" t="s" s="2">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s" s="2">
         <v>12</v>
@@ -847,409 +847,409 @@
         <v>12</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E23" t="s" s="2">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C24" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D24" t="s" s="2">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="E24" t="s" s="2">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D25" t="s" s="2">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s" s="2">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C26" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="E26" t="s" s="2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C27" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D27" t="s" s="2">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="E27" t="s" s="2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C28" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D28" t="s" s="2">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="E28" t="s" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="E29" t="s" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C30" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D30" t="s" s="2">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E30" t="s" s="2">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C31" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D31" t="s" s="2">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E31" t="s" s="2">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C32" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D32" t="s" s="2">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="E32" t="s" s="2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="C33" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D33" t="s" s="2">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="E33" t="s" s="2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D34" t="s" s="2">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E34" t="s" s="2">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C35" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D35" t="s" s="2">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E35" t="s" s="2">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="B36" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B36" t="s" s="2">
-        <v>62</v>
-      </c>
       <c r="C36" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D36" t="s" s="2">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="E36" t="s" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C37" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D37" t="s" s="2">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="E37" t="s" s="2">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C38" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D38" t="s" s="2">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E38" t="s" s="2">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C39" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D39" t="s" s="2">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E39" t="s" s="2">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C40" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D40" t="s" s="2">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E40" t="s" s="2">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D41" t="s" s="2">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E41" t="s" s="2">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C42" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D42" t="s" s="2">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E42" t="s" s="2">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C43" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D43" t="s" s="2">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E43" t="s" s="2">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C44" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D44" t="s" s="2">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="E44" t="s" s="2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -1259,16 +1259,16 @@
         <v>72</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C45" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D45" t="s" s="2">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="E45" t="s" s="2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -1278,16 +1278,16 @@
         <v>73</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C46" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D46" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E46" t="s" s="2">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -1297,16 +1297,16 @@
         <v>74</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C47" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D47" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E47" t="s" s="2">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -1316,16 +1316,16 @@
         <v>75</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C48" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D48" t="s" s="2">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E48" t="s" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -1335,16 +1335,16 @@
         <v>76</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C49" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D49" t="s" s="2">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="E49" t="s" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -1354,16 +1354,16 @@
         <v>77</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="C50" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D50" t="s" s="2">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="E50" t="s" s="2">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -1373,16 +1373,16 @@
         <v>79</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="C51" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D51" t="s" s="2">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="E51" t="s" s="2">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -1392,16 +1392,16 @@
         <v>80</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="C52" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D52" t="s" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E52" t="s" s="2">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -1411,16 +1411,16 @@
         <v>81</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="C53" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D53" t="s" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E53" t="s" s="2">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -1430,16 +1430,16 @@
         <v>82</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C54" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D54" t="s" s="2">
-        <v>78</v>
+        <v>22</v>
       </c>
       <c r="E54" t="s" s="2">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -1449,16 +1449,16 @@
         <v>83</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C55" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D55" t="s" s="2">
-        <v>78</v>
+        <v>22</v>
       </c>
       <c r="E55" t="s" s="2">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -1468,16 +1468,16 @@
         <v>84</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C56" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D56" t="s" s="2">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="E56" t="s" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -1487,16 +1487,16 @@
         <v>85</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C57" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D57" t="s" s="2">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="E57" t="s" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -1506,92 +1506,92 @@
         <v>86</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="C58" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D58" t="s" s="2">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="E58" t="s" s="2">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="C59" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D59" t="s" s="2">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="E59" t="s" s="2">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="C60" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D60" t="s" s="2">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="E60" t="s" s="2">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="C61" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D61" t="s" s="2">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="E61" t="s" s="2">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="B62" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="B62" t="s" s="2">
-        <v>47</v>
-      </c>
       <c r="C62" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D62" t="s" s="2">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="E62" t="s" s="2">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -1601,16 +1601,16 @@
         <v>92</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D63" t="s" s="2">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="E63" t="s" s="2">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
@@ -1620,16 +1620,16 @@
         <v>93</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C64" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D64" t="s" s="2">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E64" t="s" s="2">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
@@ -1639,16 +1639,16 @@
         <v>94</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D65" t="s" s="2">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E65" t="s" s="2">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
@@ -1658,16 +1658,16 @@
         <v>95</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D66" t="s" s="2">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E66" t="s" s="2">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -1677,16 +1677,16 @@
         <v>96</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D67" t="s" s="2">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="E67" t="s" s="2">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -1696,16 +1696,16 @@
         <v>97</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D68" t="s" s="2">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E68" t="s" s="2">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -1715,16 +1715,16 @@
         <v>98</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D69" t="s" s="2">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E69" t="s" s="2">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -1734,16 +1734,16 @@
         <v>99</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D70" t="s" s="2">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E70" t="s" s="2">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -1753,16 +1753,16 @@
         <v>100</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="C71" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D71" t="s" s="2">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E71" t="s" s="2">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -1772,16 +1772,16 @@
         <v>101</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C72" t="s" s="2">
         <v>8</v>
       </c>
       <c r="D72" t="s" s="2">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E72" t="s" s="2">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
@@ -1791,16 +1791,16 @@
         <v>102</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="C73" t="s" s="2">
         <v>12</v>
       </c>
       <c r="D73" t="s" s="2">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E73" t="s" s="2">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>

</xml_diff>